<commit_message>
Sector in investors (#1268)
* Added sector in Investors form, show and upload

* Updated all excel files for investors to have sector

* Updated portfolio companies xl
</commit_message>
<xml_diff>
--- a/public/sample_uploads/allocate_account_entries/investors.xlsx
+++ b/public/sample_uploads/allocate_account_entries/investors.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
-    <author>Author</author>
+    <author>Unknown Author</author>
   </authors>
   <commentList>
     <comment ref="A1" authorId="0">
@@ -153,7 +153,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F1" authorId="0">
+    <comment ref="G1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -182,7 +182,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="25">
   <si>
     <t xml:space="preserve">Name *</t>
   </si>
@@ -197,6 +197,9 @@
   </si>
   <si>
     <t xml:space="preserve">Category *</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sector</t>
   </si>
   <si>
     <t xml:space="preserve">City</t>
@@ -263,7 +266,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -308,13 +311,6 @@
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -385,7 +381,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -406,11 +402,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -538,16 +530,16 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F1048576"/>
-  <sheetFormatPr defaultColWidth="9.30859375" defaultRowHeight="18" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:G1048576"/>
+  <sheetFormatPr defaultColWidth="9.30859375" defaultRowHeight="18" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.09"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="7.25"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24.18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="8.46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="7.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16383" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="7.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -569,105 +561,113 @@
       <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="18" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="18" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="18" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="18" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>16</v>
-      </c>
       <c r="E6" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="6" t="s">
         <v>20</v>
       </c>
+      <c r="C7" s="4" t="s">
+        <v>21</v>
+      </c>
       <c r="E7" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>